<commit_message>
Diplomarbeit-Formular: finale Themenaufteilung eingetragen
Patrick: Recht & Vereinsführung, Gesamtarchitektur & Projektleitung,
Sicherheit & Datenschutz, Rechnungsdesign. Alexander Brunner: Hardware
& Firmware der P1-Ausleseeinheit. Fabian Amlacher: Web-Frontend/-Backend,
Serverinfrastruktur, EDA-Datenimport, Abrechnungslogik inkl. SEPA-Export.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Projektkoordination &amp; Vereinsführung (Obmann); Gesamtarchitektur der Plattform Strom für alle</t>
+          <t>Vereinsführung, Netzbetreiber-Vertrag &amp; Tarife (Obmann); Gesamtarchitektur &amp; Projektleitung; Sicherheit &amp; Datenschutz der Plattform Strom für alle</t>
         </is>
       </c>
     </row>
@@ -670,8 +670,8 @@
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Infrastruktur, Frontend, ESP32-Firmware-Pipeline
-Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; EDA-Datenimport, Abrechnungslogik</t>
+          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Web-Frontend &amp; -Backend, Serverinfrastruktur (Docker, Datenbank, Backup), EDA-Datenimport, Abrechnungslogik (Rechnungserstellung, SEPA-Lastschrift)
+Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; Hardware &amp; Firmware der selbst gebauten P1-Ausleseeinheit (Platine, 3D-Druck, P1-Schnittstelle, MQTT, WLAN)</t>
         </is>
       </c>
     </row>
@@ -776,9 +776,9 @@
       <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung) auf Basis von PostgreSQL/TimescaleDB, PHP, nginx/Traefik und Docker. Gemeinsam wird untersucht, wie Echtzeit-Messdaten (ESP32/P1-Schnittstelle) und die offiziellen EDA-Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten technisch und organisatorisch umgesetzt wird.
-Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz, Tarifgestaltung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung, rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG) und steuerlicher Beratung.
-Fabian Amlacher (Kassier): Aufbau der Serverinfrastruktur (Docker, Traefik, MQTT/Mosquitto); Entwicklung des Frontends der Plattform; Entwicklung und Test der ESP32-Firmware zum Auslesen der P1-Schnittstelle intelligenter Stromzähler sowie der MQTT-Datenpipeline von der Messstelle bis in die Datenbank.
-Alexander Brunner: Entwicklung der Importlogik für die manuellen EDA-XLSX-Exporte des Netzbetreibers (rechtliche Verrechnungsdatenbasis) sowie der Abrechnungslogik der Plattform (quartalsweise/jährliche Verrechnung von Bezug und Einspeisung je Mitglied).</t>
+Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); Sicherheit &amp; Datenschutz (DSGVO, Verschlüsselung, Zugriffsschutz, Demo-Modus) in enger Abstimmung mit Fabian (Webseite) und Alexander (Ausleseeinheit); rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
+Fabian Amlacher (Kassier): Aufbau der Serverinfrastruktur (Docker, Traefik, MQTT/Mosquitto, PostgreSQL/TimescaleDB, Backup); Entwicklung von Frontend und Backend der Plattform (Mitgliederverwaltung, Live-Anzeige); Import der manuellen EDA-XLSX-Exporte des Netzbetreibers und Zuordnung der Verbrauchs-/Einspeisewerte je Zählpunkt in der Datenbank; Abrechnungslogik inkl. Rechnungserstellung über einen LaTeX-zu-PDF-Service und Erstellung der SEPA-Lastschrift-Datei für den Bankeinzug.
+Alexander Brunner: Entwicklung von Hardware (Platinen-Design, Bauteilauswahl, 3D-Druck-Gehäuse) und Firmware (P1-Schnittstelle intelligenter Stromzähler, MQTT-Übertragung, WLAN-Setup) der selbst gebauten P1-Ausleseeinheit sowie deren Inbetriebnahme und Test.</t>
         </is>
       </c>
     </row>
@@ -832,9 +832,9 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB) sowie eine dokumentierte Gesamtarchitektur und Projektsteuerung der Plattform Strom für alle.
-Fabian Amlacher: Ein lauffähiges Frontend der Plattform sowie eine funktionierende ESP32-Firmware inklusive MQTT-Pipeline, die Echtzeit-Leistungsdaten mehrerer Zählpunkte zuverlässig in die Datenbank überträgt.
-Alexander Brunner: Ein funktionierender Import der EDA-Verrechnungsdaten sowie eine automatisierte Abrechnungslogik, die aus den importierten Viertelstundenwerten korrekte, EAG-konforme Rechnungen je Mitglied erzeugt.</t>
+          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB), eine dokumentierte Gesamtarchitektur und Projektsteuerung sowie ein datenschutz- und sicherheitskonform umgesetztes Konzept (DSGVO, Verschlüsselung, Zugriffsschutz) der Plattform Strom für alle.
+Fabian Amlacher: Ein lauffähiges Frontend und Backend der Plattform samt Serverinfrastruktur (Docker, Datenbank, Backup) sowie ein funktionierender EDA-Datenimport und eine automatisierte Abrechnungslogik inkl. Rechnungserstellung (LaTeX zu PDF) und SEPA-Lastschrift-Export.
+Alexander Brunner: Eine selbst entwickelte und gefertigte P1-Ausleseeinheit (Platine, 3D-gedrucktes Gehäuse) mit funktionierender Firmware (P1-Schnittstelle, MQTT-Übertragung, WLAN-Konfiguration), einsatzbereit bei den Mitgliedern der Pilot-EEG.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: finale Themenaufteilung eingetragen (#169)
Patrick: Recht & Vereinsführung, Gesamtarchitektur & Projektleitung,
Sicherheit & Datenschutz, Rechnungsdesign. Alexander Brunner: Hardware
& Firmware der P1-Ausleseeinheit. Fabian Amlacher: Web-Frontend/-Backend,
Serverinfrastruktur, EDA-Datenimport, Abrechnungslogik inkl. SEPA-Export.


Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Projektkoordination &amp; Vereinsführung (Obmann); Gesamtarchitektur der Plattform Strom für alle</t>
+          <t>Vereinsführung, Netzbetreiber-Vertrag &amp; Tarife (Obmann); Gesamtarchitektur &amp; Projektleitung; Sicherheit &amp; Datenschutz der Plattform Strom für alle</t>
         </is>
       </c>
     </row>
@@ -670,8 +670,8 @@
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Infrastruktur, Frontend, ESP32-Firmware-Pipeline
-Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; EDA-Datenimport, Abrechnungslogik</t>
+          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Web-Frontend &amp; -Backend, Serverinfrastruktur (Docker, Datenbank, Backup), EDA-Datenimport, Abrechnungslogik (Rechnungserstellung, SEPA-Lastschrift)
+Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; Hardware &amp; Firmware der selbst gebauten P1-Ausleseeinheit (Platine, 3D-Druck, P1-Schnittstelle, MQTT, WLAN)</t>
         </is>
       </c>
     </row>
@@ -776,9 +776,9 @@
       <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung) auf Basis von PostgreSQL/TimescaleDB, PHP, nginx/Traefik und Docker. Gemeinsam wird untersucht, wie Echtzeit-Messdaten (ESP32/P1-Schnittstelle) und die offiziellen EDA-Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten technisch und organisatorisch umgesetzt wird.
-Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz, Tarifgestaltung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung, rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG) und steuerlicher Beratung.
-Fabian Amlacher (Kassier): Aufbau der Serverinfrastruktur (Docker, Traefik, MQTT/Mosquitto); Entwicklung des Frontends der Plattform; Entwicklung und Test der ESP32-Firmware zum Auslesen der P1-Schnittstelle intelligenter Stromzähler sowie der MQTT-Datenpipeline von der Messstelle bis in die Datenbank.
-Alexander Brunner: Entwicklung der Importlogik für die manuellen EDA-XLSX-Exporte des Netzbetreibers (rechtliche Verrechnungsdatenbasis) sowie der Abrechnungslogik der Plattform (quartalsweise/jährliche Verrechnung von Bezug und Einspeisung je Mitglied).</t>
+Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); Sicherheit &amp; Datenschutz (DSGVO, Verschlüsselung, Zugriffsschutz, Demo-Modus) in enger Abstimmung mit Fabian (Webseite) und Alexander (Ausleseeinheit); rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
+Fabian Amlacher (Kassier): Aufbau der Serverinfrastruktur (Docker, Traefik, MQTT/Mosquitto, PostgreSQL/TimescaleDB, Backup); Entwicklung von Frontend und Backend der Plattform (Mitgliederverwaltung, Live-Anzeige); Import der manuellen EDA-XLSX-Exporte des Netzbetreibers und Zuordnung der Verbrauchs-/Einspeisewerte je Zählpunkt in der Datenbank; Abrechnungslogik inkl. Rechnungserstellung über einen LaTeX-zu-PDF-Service und Erstellung der SEPA-Lastschrift-Datei für den Bankeinzug.
+Alexander Brunner: Entwicklung von Hardware (Platinen-Design, Bauteilauswahl, 3D-Druck-Gehäuse) und Firmware (P1-Schnittstelle intelligenter Stromzähler, MQTT-Übertragung, WLAN-Setup) der selbst gebauten P1-Ausleseeinheit sowie deren Inbetriebnahme und Test.</t>
         </is>
       </c>
     </row>
@@ -832,9 +832,9 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB) sowie eine dokumentierte Gesamtarchitektur und Projektsteuerung der Plattform Strom für alle.
-Fabian Amlacher: Ein lauffähiges Frontend der Plattform sowie eine funktionierende ESP32-Firmware inklusive MQTT-Pipeline, die Echtzeit-Leistungsdaten mehrerer Zählpunkte zuverlässig in die Datenbank überträgt.
-Alexander Brunner: Ein funktionierender Import der EDA-Verrechnungsdaten sowie eine automatisierte Abrechnungslogik, die aus den importierten Viertelstundenwerten korrekte, EAG-konforme Rechnungen je Mitglied erzeugt.</t>
+          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB), eine dokumentierte Gesamtarchitektur und Projektsteuerung sowie ein datenschutz- und sicherheitskonform umgesetztes Konzept (DSGVO, Verschlüsselung, Zugriffsschutz) der Plattform Strom für alle.
+Fabian Amlacher: Ein lauffähiges Frontend und Backend der Plattform samt Serverinfrastruktur (Docker, Datenbank, Backup) sowie ein funktionierender EDA-Datenimport und eine automatisierte Abrechnungslogik inkl. Rechnungserstellung (LaTeX zu PDF) und SEPA-Lastschrift-Export.
+Alexander Brunner: Eine selbst entwickelte und gefertigte P1-Ausleseeinheit (Platine, 3D-gedrucktes Gehäuse) mit funktionierender Firmware (P1-Schnittstelle, MQTT-Übertragung, WLAN-Konfiguration), einsatzbereit bei den Mitgliedern der Pilot-EEG.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: Beschreibung auf Ziele statt Umsetzung fokussiert
Untersuchungsanliegen (E13) und geplantes Ergebnis (E15) beschreiben
jetzt, was erreicht werden soll, nicht mehr mit welchem konkreten
Tech-Stack (Docker, Traefik, PostgreSQL/TimescaleDB, LaTeX-zu-PDF, ...) -
das ist ja Teil der eigentlichen Diplomarbeitsarbeit und soll nicht
bereits im Anmeldeformular als fertig entschieden wirken.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -670,8 +670,8 @@
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Web-Frontend &amp; -Backend, Serverinfrastruktur (Docker, Datenbank, Backup), EDA-Datenimport, Abrechnungslogik (Rechnungserstellung, SEPA-Lastschrift)
-Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; Hardware &amp; Firmware der selbst gebauten P1-Ausleseeinheit (Platine, 3D-Druck, P1-Schnittstelle, MQTT, WLAN)</t>
+          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Plattform (Verwaltung &amp; Anzeige), Serverbetrieb, Einlesen der Verrechnungsdaten, automatisierte Abrechnung &amp; Bankeinzug
+Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; Hardware &amp; Firmware der selbst entwickelten Ausleseeinheit für die Zählerdaten</t>
         </is>
       </c>
     </row>
@@ -775,10 +775,10 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung) auf Basis von PostgreSQL/TimescaleDB, PHP, nginx/Traefik und Docker. Gemeinsam wird untersucht, wie Echtzeit-Messdaten (ESP32/P1-Schnittstelle) und die offiziellen EDA-Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten technisch und organisatorisch umgesetzt wird.
-Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); Sicherheit &amp; Datenschutz (DSGVO, Verschlüsselung, Zugriffsschutz, Demo-Modus) in enger Abstimmung mit Fabian (Webseite) und Alexander (Ausleseeinheit); rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
-Fabian Amlacher (Kassier): Aufbau der Serverinfrastruktur (Docker, Traefik, MQTT/Mosquitto, PostgreSQL/TimescaleDB, Backup); Entwicklung von Frontend und Backend der Plattform (Mitgliederverwaltung, Live-Anzeige); Import der manuellen EDA-XLSX-Exporte des Netzbetreibers und Zuordnung der Verbrauchs-/Einspeisewerte je Zählpunkt in der Datenbank; Abrechnungslogik inkl. Rechnungserstellung über einen LaTeX-zu-PDF-Service und Erstellung der SEPA-Lastschrift-Datei für den Bankeinzug.
-Alexander Brunner: Entwicklung von Hardware (Platinen-Design, Bauteilauswahl, 3D-Druck-Gehäuse) und Firmware (P1-Schnittstelle intelligenter Stromzähler, MQTT-Übertragung, WLAN-Setup) der selbst gebauten P1-Ausleseeinheit sowie deren Inbetriebnahme und Test.</t>
+          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung). Gemeinsam wird untersucht, wie Echtzeit-Messdaten der Zählpunkte und die offiziellen Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür jeweils am besten eignen, ist selbst Teil der Untersuchung.
+Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); wie Sicherheit und Datenschutz (u.a. DSGVO-Vorgaben, Zugriffsschutz) in einer solchen Plattform sinnvoll umgesetzt werden können, in enger Abstimmung mit Fabian und Alexander; rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
+Fabian Amlacher (Kassier): Wie eine zuverlässige, wartbare Serverinfrastruktur für eine solche Plattform aufgebaut werden kann; Entwicklung von Frontend und Backend (Mitgliederverwaltung, Live-Anzeige); wie die vom Netzbetreiber bereitgestellten Verrechnungsdaten automatisiert eingelesen und den richtigen Zählpunkten zugeordnet werden können; wie daraus automatisiert korrekte Rechnungen sowie ein Sammellastschrift-Auftrag für den Bankeinzug erzeugt werden können.
+Alexander Brunner: Entwicklung einer eigenen Hardware (Platine, Bauteilauswahl, Gehäuse) zum Auslesen der P1-Schnittstelle intelligenter Stromzähler sowie der dazugehörigen Firmware zur zuverlässigen, sicheren Übertragung der Messdaten; Inbetriebnahme und Test bei realen Mitgliedern.</t>
         </is>
       </c>
     </row>
@@ -832,9 +832,9 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB), eine dokumentierte Gesamtarchitektur und Projektsteuerung sowie ein datenschutz- und sicherheitskonform umgesetztes Konzept (DSGVO, Verschlüsselung, Zugriffsschutz) der Plattform Strom für alle.
-Fabian Amlacher: Ein lauffähiges Frontend und Backend der Plattform samt Serverinfrastruktur (Docker, Datenbank, Backup) sowie ein funktionierender EDA-Datenimport und eine automatisierte Abrechnungslogik inkl. Rechnungserstellung (LaTeX zu PDF) und SEPA-Lastschrift-Export.
-Alexander Brunner: Eine selbst entwickelte und gefertigte P1-Ausleseeinheit (Platine, 3D-gedrucktes Gehäuse) mit funktionierender Firmware (P1-Schnittstelle, MQTT-Übertragung, WLAN-Konfiguration), einsatzbereit bei den Mitgliedern der Pilot-EEG.</t>
+          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB), eine dokumentierte Gesamtarchitektur und Projektsteuerung sowie ein datenschutz- und sicherheitskonform umgesetztes Konzept der Plattform Strom für alle.
+Fabian Amlacher: Eine lauffähige Plattform (Frontend, Backend, Serverbetrieb), die die Verrechnungsdaten des Netzbetreibers automatisiert einliest und daraus korrekte Rechnungen sowie einen Sammellastschrift-Auftrag für den Bankeinzug erzeugt.
+Alexander Brunner: Eine selbst entwickelte und gefertigte Ausleseeinheit (Platine, Gehäuse) mit funktionierender Firmware, die die Messdaten intelligenter Stromzähler zuverlässig überträgt, einsatzbereit bei den Mitgliedern der Pilot-EEG.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: Beschreibung auf Ziele statt Umsetzung fokussiert (#170)
Untersuchungsanliegen (E13) und geplantes Ergebnis (E15) beschreiben
jetzt, was erreicht werden soll, nicht mehr mit welchem konkreten
Tech-Stack (Docker, Traefik, PostgreSQL/TimescaleDB, LaTeX-zu-PDF, ...) -
das ist ja Teil der eigentlichen Diplomarbeitsarbeit und soll nicht
bereits im Anmeldeformular als fertig entschieden wirken.


Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -670,8 +670,8 @@
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Web-Frontend &amp; -Backend, Serverinfrastruktur (Docker, Datenbank, Backup), EDA-Datenimport, Abrechnungslogik (Rechnungserstellung, SEPA-Lastschrift)
-Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; Hardware &amp; Firmware der selbst gebauten P1-Ausleseeinheit (Platine, 3D-Druck, P1-Schnittstelle, MQTT, WLAN)</t>
+          <t>Fabian Amlacher (Abteilung: Elektrotechnik) – Kassier; Plattform (Verwaltung &amp; Anzeige), Serverbetrieb, Einlesen der Verrechnungsdaten, automatisierte Abrechnung &amp; Bankeinzug
+Alexander Brunner (Abteilung: Elektrotechnik) – Gründungsmitglied; Hardware &amp; Firmware der selbst entwickelten Ausleseeinheit für die Zählerdaten</t>
         </is>
       </c>
     </row>
@@ -775,10 +775,10 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung) auf Basis von PostgreSQL/TimescaleDB, PHP, nginx/Traefik und Docker. Gemeinsam wird untersucht, wie Echtzeit-Messdaten (ESP32/P1-Schnittstelle) und die offiziellen EDA-Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten technisch und organisatorisch umgesetzt wird.
-Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); Sicherheit &amp; Datenschutz (DSGVO, Verschlüsselung, Zugriffsschutz, Demo-Modus) in enger Abstimmung mit Fabian (Webseite) und Alexander (Ausleseeinheit); rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
-Fabian Amlacher (Kassier): Aufbau der Serverinfrastruktur (Docker, Traefik, MQTT/Mosquitto, PostgreSQL/TimescaleDB, Backup); Entwicklung von Frontend und Backend der Plattform (Mitgliederverwaltung, Live-Anzeige); Import der manuellen EDA-XLSX-Exporte des Netzbetreibers und Zuordnung der Verbrauchs-/Einspeisewerte je Zählpunkt in der Datenbank; Abrechnungslogik inkl. Rechnungserstellung über einen LaTeX-zu-PDF-Service und Erstellung der SEPA-Lastschrift-Datei für den Bankeinzug.
-Alexander Brunner: Entwicklung von Hardware (Platinen-Design, Bauteilauswahl, 3D-Druck-Gehäuse) und Firmware (P1-Schnittstelle intelligenter Stromzähler, MQTT-Übertragung, WLAN-Setup) der selbst gebauten P1-Ausleseeinheit sowie deren Inbetriebnahme und Test.</t>
+          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung). Gemeinsam wird untersucht, wie Echtzeit-Messdaten der Zählpunkte und die offiziellen Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür jeweils am besten eignen, ist selbst Teil der Untersuchung.
+Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); wie Sicherheit und Datenschutz (u.a. DSGVO-Vorgaben, Zugriffsschutz) in einer solchen Plattform sinnvoll umgesetzt werden können, in enger Abstimmung mit Fabian und Alexander; rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
+Fabian Amlacher (Kassier): Wie eine zuverlässige, wartbare Serverinfrastruktur für eine solche Plattform aufgebaut werden kann; Entwicklung von Frontend und Backend (Mitgliederverwaltung, Live-Anzeige); wie die vom Netzbetreiber bereitgestellten Verrechnungsdaten automatisiert eingelesen und den richtigen Zählpunkten zugeordnet werden können; wie daraus automatisiert korrekte Rechnungen sowie ein Sammellastschrift-Auftrag für den Bankeinzug erzeugt werden können.
+Alexander Brunner: Entwicklung einer eigenen Hardware (Platine, Bauteilauswahl, Gehäuse) zum Auslesen der P1-Schnittstelle intelligenter Stromzähler sowie der dazugehörigen Firmware zur zuverlässigen, sicheren Übertragung der Messdaten; Inbetriebnahme und Test bei realen Mitgliedern.</t>
         </is>
       </c>
     </row>
@@ -832,9 +832,9 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB), eine dokumentierte Gesamtarchitektur und Projektsteuerung sowie ein datenschutz- und sicherheitskonform umgesetztes Konzept (DSGVO, Verschlüsselung, Zugriffsschutz) der Plattform Strom für alle.
-Fabian Amlacher: Ein lauffähiges Frontend und Backend der Plattform samt Serverinfrastruktur (Docker, Datenbank, Backup) sowie ein funktionierender EDA-Datenimport und eine automatisierte Abrechnungslogik inkl. Rechnungserstellung (LaTeX zu PDF) und SEPA-Lastschrift-Export.
-Alexander Brunner: Eine selbst entwickelte und gefertigte P1-Ausleseeinheit (Platine, 3D-gedrucktes Gehäuse) mit funktionierender Firmware (P1-Schnittstelle, MQTT-Übertragung, WLAN-Konfiguration), einsatzbereit bei den Mitgliedern der Pilot-EEG.</t>
+          <t>Patrick Ropper: Eine im Verein eingetragene und beim Netzbetreiber aktive Energiegemeinschaft (Statuten, Mitgliederverträge, Tarifblatt, AGB), eine dokumentierte Gesamtarchitektur und Projektsteuerung sowie ein datenschutz- und sicherheitskonform umgesetztes Konzept der Plattform Strom für alle.
+Fabian Amlacher: Eine lauffähige Plattform (Frontend, Backend, Serverbetrieb), die die Verrechnungsdaten des Netzbetreibers automatisiert einliest und daraus korrekte Rechnungen sowie einen Sammellastschrift-Auftrag für den Bankeinzug erzeugt.
+Alexander Brunner: Eine selbst entwickelte und gefertigte Ausleseeinheit (Platine, Gehäuse) mit funktionierender Firmware, die die Messdaten intelligenter Stromzähler zuverlässig überträgt, einsatzbereit bei den Mitgliedern der Pilot-EEG.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: EEG-Gründung als offene Aufgabe statt Faktum
Ausgangslage (E12) und Meilensteine (E16) behaupteten bisher, die
Pilot-EEG sei bereits gegründet und der Netzbetreiber-Vertrag bereits
abgeschlossen. Das widerspricht Patricks Themenstellung (Recht &
Vereinsführung: den Weg zur Gründung einer Energiegemeinschaft selbst
zeigen) - beides steht jetzt als offener Meilenstein statt als
abgeschlossene Tatsache. Zusätzlich in E13 die DSGVO-Detailaufzählung
bei "Sicherheit & Datenschutz" entfernt - das Portal braucht nur das
Thema, nicht den Umsetzungsplan.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -748,7 +748,7 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>In Kärnten entstehen im Zuge der Energiewende laufend neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis wurde die Pilot-EEG „Strompool Feldkirchen Süd-West“ bereits gegründet.</t>
+          <t>In Kärnten entstehen im Zuge der Energiewende laufend neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis soll die Pilot-EEG „Strompool Feldkirchen Süd-West“ gegründet und aufgebaut werden.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung). Gemeinsam wird untersucht, wie Echtzeit-Messdaten der Zählpunkte und die offiziellen Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür jeweils am besten eignen, ist selbst Teil der Untersuchung.
-Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); wie Sicherheit und Datenschutz (u.a. DSGVO-Vorgaben, Zugriffsschutz) in einer solchen Plattform sinnvoll umgesetzt werden können, in enger Abstimmung mit Fabian und Alexander; rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
+Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); wie Sicherheit und Datenschutz in einer solchen Plattform sinnvoll umgesetzt werden können, in enger Abstimmung mit Fabian und Alexander; rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
 Fabian Amlacher (Kassier): Wie eine zuverlässige, wartbare Serverinfrastruktur für eine solche Plattform aufgebaut werden kann; Entwicklung von Frontend und Backend (Mitgliederverwaltung, Live-Anzeige); wie die vom Netzbetreiber bereitgestellten Verrechnungsdaten automatisiert eingelesen und den richtigen Zählpunkten zugeordnet werden können; wie daraus automatisiert korrekte Rechnungen sowie ein Sammellastschrift-Auftrag für den Bankeinzug erzeugt werden können.
 Alexander Brunner: Entwicklung einer eigenen Hardware (Platine, Bauteilauswahl, Gehäuse) zum Auslesen der P1-Schnittstelle intelligenter Stromzähler sowie der dazugehörigen Firmware zur zuverlässigen, sicheren Übertragung der Messdaten; Inbetriebnahme und Test bei realen Mitgliedern.</t>
         </is>
@@ -857,12 +857,13 @@
       <c r="D16" s="10" t="n"/>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>(Portal akzeptiert nur zukünftige Termine – bereits erledigte Schritte wie Vereinsgründung, KNG-Vertrag etc. sind daher hier nicht mehr gelistet.)
+          <t>❓ Datum: Vereinsgründung &amp; Statuten der Pilot-EEG
+❓ Datum: Vertragsabschluss mit dem Netzbetreiber (KNG)
 ❓ Datum: Zwischenpräsentation der Diplomarbeit
-❓ Datum: Fertigstellung Paket 2 – Abrechnung (pdflatex-Bug &amp; EDA-Upload-Fehler beheben, Ende-zu-Ende-Billing)
+❓ Datum: Fertigstellung Paket 2 – Abrechnung
 ❓ Datum: Fertigstellung Paket 3 – Backup-Monitor für Admins
 ❓ Datum: SEPA-Lastschrift – Creditor-ID-Antrag abschließen
-❓ Datum: Klärung KNG-Datenfreigabe-Prozess (Sammel-Vollmacht vs. Einzel-Login je Mitglied)
+❓ Datum: Klärung KNG-Datenfreigabe-Prozess
 ❓ Datum: Dokumentation &amp; Abschluss
 ❓ Datum: Abgabe der Diplomarbeit (siehe Zeile 6)</t>
         </is>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: EEG-Gründung als offene Aufgabe statt Faktum (#171)
Ausgangslage (E12) und Meilensteine (E16) behaupteten bisher, die
Pilot-EEG sei bereits gegründet und der Netzbetreiber-Vertrag bereits
abgeschlossen. Das widerspricht Patricks Themenstellung (Recht &
Vereinsführung: den Weg zur Gründung einer Energiegemeinschaft selbst
zeigen) - beides steht jetzt als offener Meilenstein statt als
abgeschlossene Tatsache. Zusätzlich in E13 die DSGVO-Detailaufzählung
bei "Sicherheit & Datenschutz" entfernt - das Portal braucht nur das
Thema, nicht den Umsetzungsplan.


Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -748,7 +748,7 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>In Kärnten entstehen im Zuge der Energiewende laufend neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis wurde die Pilot-EEG „Strompool Feldkirchen Süd-West“ bereits gegründet.</t>
+          <t>In Kärnten entstehen im Zuge der Energiewende laufend neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis soll die Pilot-EEG „Strompool Feldkirchen Süd-West“ gegründet und aufgebaut werden.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung). Gemeinsam wird untersucht, wie Echtzeit-Messdaten der Zählpunkte und die offiziellen Verrechnungsdaten des Netzbetreibers sauber getrennt und für Visualisierung bzw. rechtssichere Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür jeweils am besten eignen, ist selbst Teil der Untersuchung.
-Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); wie Sicherheit und Datenschutz (u.a. DSGVO-Vorgaben, Zugriffsschutz) in einer solchen Plattform sinnvoll umgesetzt werden können, in enger Abstimmung mit Fabian und Alexander; rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
+Patrick Ropper (Obmann): Projektkoordination und Entscheidungsfindung im Team; Gründung und laufende Führung der Pilot-EEG (Statuten, Vertrag mit dem Netzbetreiber KNG-Kärnten Netz inkl. Festlegung des Aufteilungsschlüssels, Tarifgestaltung, steuerliche Beratung); Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); wie Sicherheit und Datenschutz in einer solchen Plattform sinnvoll umgesetzt werden können, in enger Abstimmung mit Fabian und Alexander; rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
 Fabian Amlacher (Kassier): Wie eine zuverlässige, wartbare Serverinfrastruktur für eine solche Plattform aufgebaut werden kann; Entwicklung von Frontend und Backend (Mitgliederverwaltung, Live-Anzeige); wie die vom Netzbetreiber bereitgestellten Verrechnungsdaten automatisiert eingelesen und den richtigen Zählpunkten zugeordnet werden können; wie daraus automatisiert korrekte Rechnungen sowie ein Sammellastschrift-Auftrag für den Bankeinzug erzeugt werden können.
 Alexander Brunner: Entwicklung einer eigenen Hardware (Platine, Bauteilauswahl, Gehäuse) zum Auslesen der P1-Schnittstelle intelligenter Stromzähler sowie der dazugehörigen Firmware zur zuverlässigen, sicheren Übertragung der Messdaten; Inbetriebnahme und Test bei realen Mitgliedern.</t>
         </is>
@@ -857,12 +857,13 @@
       <c r="D16" s="10" t="n"/>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>(Portal akzeptiert nur zukünftige Termine – bereits erledigte Schritte wie Vereinsgründung, KNG-Vertrag etc. sind daher hier nicht mehr gelistet.)
+          <t>❓ Datum: Vereinsgründung &amp; Statuten der Pilot-EEG
+❓ Datum: Vertragsabschluss mit dem Netzbetreiber (KNG)
 ❓ Datum: Zwischenpräsentation der Diplomarbeit
-❓ Datum: Fertigstellung Paket 2 – Abrechnung (pdflatex-Bug &amp; EDA-Upload-Fehler beheben, Ende-zu-Ende-Billing)
+❓ Datum: Fertigstellung Paket 2 – Abrechnung
 ❓ Datum: Fertigstellung Paket 3 – Backup-Monitor für Admins
 ❓ Datum: SEPA-Lastschrift – Creditor-ID-Antrag abschließen
-❓ Datum: Klärung KNG-Datenfreigabe-Prozess (Sammel-Vollmacht vs. Einzel-Login je Mitglied)
+❓ Datum: Klärung KNG-Datenfreigabe-Prozess
 ❓ Datum: Dokumentation &amp; Abschluss
 ❓ Datum: Abgabe der Diplomarbeit (siehe Zeile 6)</t>
         </is>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: korrekten Namen der Energiegemeinschaft verwendet
Statt "Energiegemeinschaft Strompool Feldkirchen Südwest" (verkürzt/falsche
Schreibweise) jetzt durchgehend der tatsächliche Name: "Erneuerbare-Energie-
Gemeinschaft Strompool Feldkirchen Süd-West" (Thema, Ausgangslage Variante B,
Zielsetzung; im Untersuchungsanliegen bleibt aus Platzgründen die bereits
etablierte Abkürzung "EEG", jetzt mit korrektem Süd-West statt Südwest).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Strom für alle - Entwicklung einer digitalen Plattform samt Ausleseeinheit für Echtzeit-Verbrauchsanzeige und automatisierte Abrechnung für die Energiegemeinschaft Strompool Feldkirchen Südwest</t>
+          <t>Strom für alle - Entwicklung einer Plattform samt Ausleseeinheit für Echtzeit-Verbrauchsanzeige und automatisierte Abrechnung für die Erneuerbare-Energie-Gemeinschaft Strompool Feldkirchen Süd-West</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>In Kärnten entstehen im Zuge der Energiewende neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis soll die Energiegemeinschaft Strompool Feldkirchen Südwest gegründet und aufgebaut werden.</t>
+          <t>In Kärnten entstehen neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis soll die Erneuerbare-Energie-Gemeinschaft Strompool Feldkirchen Süd-West gegründet und aufgebaut werden.</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung), mit Pilotbetrieb bei der EEG Strompool Feldkirchen Südwest. Gemeinsam wird untersucht, wie Zählerdaten technisch zuverlässig ausgelesen werden können (z. B. über die P1-Schnittstelle oder optisch/Infrarot), wie diese Echtzeit-Messdaten und die Verrechnungsdaten des Netzbetreibers für Visualisierung bzw. Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür am besten eignen, ist selbst Teil der Untersuchung.
+          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung), mit Pilotbetrieb bei der EEG Strompool Feldkirchen Süd-West. Gemeinsam wird untersucht, wie Zählerdaten technisch zuverlässig ausgelesen werden können (z. B. über die P1-Schnittstelle oder optisch/Infrarot), wie diese Echtzeit-Messdaten und die Verrechnungsdaten des Netzbetreibers für Visualisierung bzw. Abrechnung genutzt werden können, sowie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür am besten eignen, ist selbst Teil der Untersuchung.
 Patrick Ropper: Wie ein Verein gegründet und geführt wird (Statuten, Organe, Ablauf); welche Vereinbarungen mit dem Netzbetreiber (voraussichtlich Kärnten Netz) für eine Energiegemeinschaft nötig sind, inkl. Tarifgestaltung und Aufteilungsschlüssel; Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); welche rechtlichen Datenschutz-Anforderungen (DSGVO) gelten und wie sie in einer Datenschutzerklärung dokumentiert werden (technische Umsetzung der Datentrennung: Fabian); rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
 Fabian Amlacher: Wie die in der Energiegemeinschaft tatsächlich verfügbare Leistung in Echtzeit sichtbar gemacht werden kann, statt erst am Folgetag wie bei den Netzbetreiber-Daten; wie eine zuverlässige Serverinfrastruktur dafür aufgebaut werden kann; Entwicklung von Frontend und Backend (Mitgliederverwaltung, Live-Anzeige); technische Umsetzung der Datentrennung und sicheren Datenverarbeitung; wie die Verrechnungsdaten des Netzbetreibers automatisiert eingelesen und den richtigen Zählpunkten zugeordnet werden können; wie daraus automatisiert korrekte Rechnungen samt Sammellastschrift-Auftrag für den Bankeinzug erzeugt werden können.
 Alexander Brunner: Entwicklung einer eigenen Hardware (Platine, Bauteilauswahl, Gehäuse) zur Auslesung der Zählerdaten – welche Schnittstelle (P1 oder optisch/Infrarot) sich dafür am besten eignet, ist Teil der Untersuchung – sowie der dazugehörigen Firmware zur zuverlässigen, sicheren Übertragung der Messdaten; Inbetriebnahme und Test bei realen Mitgliedern.</t>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Ziel ist eine funktionsfähige, mandantenfähige Plattform „Strom für alle“, die die Energiegemeinschaft (EEG) Strompool Feldkirchen Südwest als Pilotprojekt abbildet: von der Mitgliederverwaltung über die automatisierte Abrechnung bis zur Echtzeit-Visualisierung der verfügbaren Energie. Die EEG soll im laufenden Betrieb funktionieren und als Vorlage für weitere Energiegemeinschaften dienen.</t>
+          <t>Ziel ist eine mandantenfähige Plattform „Strom für alle“, die die Erneuerbare-Energie-Gemeinschaft (EEG) Strompool Feldkirchen Süd-West als Pilotprojekt abbildet: von der Mitgliederverwaltung über die automatisierte Abrechnung bis zur Echtzeit-Visualisierung der verfügbaren Energie. Die EEG soll im Betrieb funktionieren und als Vorlage für weitere Energiegemeinschaften dienen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diplomarbeit-Formular: korrekten Namen der Energiegemeinschaft verwendet (#174)
Statt "Energiegemeinschaft Strompool Feldkirchen Südwest" (verkürzt/falsche
Schreibweise) jetzt durchgehend der tatsächliche Name: "Erneuerbare-Energie-
Gemeinschaft Strompool Feldkirchen Süd-West" (Thema, Ausgangslage Variante B,
Zielsetzung; im Untersuchungsanliegen bleibt aus Platzgründen die bereits
etablierte Abkürzung "EEG", jetzt mit korrektem Süd-West statt Südwest).


Claude-Session: https://claude.ai/code/session_018tQA89moVaV9JqQnbGqM3Y

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
+++ b/docs/diplomarbeit/Diplomarbeit_ABA_Eintragung.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Strom für alle - Entwicklung einer digitalen Plattform samt Ausleseeinheit für Echtzeit-Verbrauchsanzeige und automatisierte Abrechnung für die Energiegemeinschaft Strompool Feldkirchen Südwest</t>
+          <t>Strom für alle - Entwicklung einer Plattform samt Ausleseeinheit für Echtzeit-Verbrauchsanzeige und automatisierte Abrechnung für die Erneuerbare-Energie-Gemeinschaft Strompool Feldkirchen Süd-West</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>In Kärnten entstehen im Zuge der Energiewende neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis soll die Energiegemeinschaft Strompool Feldkirchen Südwest gegründet und aufgebaut werden.</t>
+          <t>In Kärnten entstehen neue Energiegemeinschaften (EEGs), doch es fehlt an einer leistbaren, mandantenfähigen Software zur Verwaltung von Mitgliedern, Zählpunkten, Tarifen und Abrechnung. Bestehende Lösungen sind für kleine regionale EEGs zu teuer oder zu komplex. Als Praxisbasis soll die Erneuerbare-Energie-Gemeinschaft Strompool Feldkirchen Süd-West gegründet und aufgebaut werden.</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung), mit Pilotbetrieb bei der EEG Strompool Feldkirchen Südwest. Gemeinsam wird untersucht, wie Zählerdaten technisch zuverlässig ausgelesen werden können (z. B. über die P1-Schnittstelle oder optisch/Infrarot), wie diese Echtzeit-Messdaten und die Verrechnungsdaten des Netzbetreibers für Visualisierung bzw. Abrechnung genutzt werden können, sowie wie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür am besten eignen, ist selbst Teil der Untersuchung.
+          <t>Gemeinsam: Aufbau der Plattform „Strom für alle“ – einer mandantenfähigen Webanwendung zur Verwaltung mehrerer Energiegemeinschaften (Mitglieder, Zählpunkte, Verträge, Tarife, Abrechnung), mit Pilotbetrieb bei der EEG Strompool Feldkirchen Süd-West. Gemeinsam wird untersucht, wie Zählerdaten technisch zuverlässig ausgelesen werden können (z. B. über die P1-Schnittstelle oder optisch/Infrarot), wie diese Echtzeit-Messdaten und die Verrechnungsdaten des Netzbetreibers für Visualisierung bzw. Abrechnung genutzt werden können, sowie eine EAG-/ElWOG-konforme, dynamische Verteilung nach Viertelstundenwerten organisatorisch und technisch umgesetzt werden kann – welche Architektur, Werkzeuge und Verfahren sich dafür am besten eignen, ist selbst Teil der Untersuchung.
 Patrick Ropper: Wie ein Verein gegründet und geführt wird (Statuten, Organe, Ablauf); welche Vereinbarungen mit dem Netzbetreiber (voraussichtlich Kärnten Netz) für eine Energiegemeinschaft nötig sind, inkl. Tarifgestaltung und Aufteilungsschlüssel; Gesamtarchitektur der Plattform sowie Schnittstelle zwischen technischer Umsetzung und rechtlichen Vorgaben (VerG, ElWOG, EAG, UStG); welche rechtlichen Datenschutz-Anforderungen (DSGVO) gelten und wie sie in einer Datenschutzerklärung dokumentiert werden (technische Umsetzung der Datentrennung: Fabian); rechtlich vorgeschriebener Rechnungsinhalt und Rechnungsdesign.
 Fabian Amlacher: Wie die in der Energiegemeinschaft tatsächlich verfügbare Leistung in Echtzeit sichtbar gemacht werden kann, statt erst am Folgetag wie bei den Netzbetreiber-Daten; wie eine zuverlässige Serverinfrastruktur dafür aufgebaut werden kann; Entwicklung von Frontend und Backend (Mitgliederverwaltung, Live-Anzeige); technische Umsetzung der Datentrennung und sicheren Datenverarbeitung; wie die Verrechnungsdaten des Netzbetreibers automatisiert eingelesen und den richtigen Zählpunkten zugeordnet werden können; wie daraus automatisiert korrekte Rechnungen samt Sammellastschrift-Auftrag für den Bankeinzug erzeugt werden können.
 Alexander Brunner: Entwicklung einer eigenen Hardware (Platine, Bauteilauswahl, Gehäuse) zur Auslesung der Zählerdaten – welche Schnittstelle (P1 oder optisch/Infrarot) sich dafür am besten eignet, ist Teil der Untersuchung – sowie der dazugehörigen Firmware zur zuverlässigen, sicheren Übertragung der Messdaten; Inbetriebnahme und Test bei realen Mitgliedern.</t>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Ziel ist eine funktionsfähige, mandantenfähige Plattform „Strom für alle“, die die Energiegemeinschaft (EEG) Strompool Feldkirchen Südwest als Pilotprojekt abbildet: von der Mitgliederverwaltung über die automatisierte Abrechnung bis zur Echtzeit-Visualisierung der verfügbaren Energie. Die EEG soll im laufenden Betrieb funktionieren und als Vorlage für weitere Energiegemeinschaften dienen.</t>
+          <t>Ziel ist eine mandantenfähige Plattform „Strom für alle“, die die Erneuerbare-Energie-Gemeinschaft (EEG) Strompool Feldkirchen Süd-West als Pilotprojekt abbildet: von der Mitgliederverwaltung über die automatisierte Abrechnung bis zur Echtzeit-Visualisierung der verfügbaren Energie. Die EEG soll im Betrieb funktionieren und als Vorlage für weitere Energiegemeinschaften dienen.</t>
         </is>
       </c>
     </row>

</xml_diff>